<commit_message>
Reframe: every conversion off Exhibit B is a win, regardless of award method
A sole-source or emergency award is still an awarded contract - justified,
documented, with negotiated terms and an audit trail. Maverick spend is the
absence of a contract vehicle. Leaving Exhibit B is the win; the method used
to award the contract is a separate question.

- Drops the pass/fail "Competitive?" column from the proof table in favour of
  a factual "Award Method" column (BID / SOLE SOURCE / EMERGENCY).
- Removes the amber warning styling that read the two non-bid awards as
  deficient.
- Summary now states all 8 are wins and reports the method mix as context
  rather than as a second gate to clear.

Figures unchanged: 8 items, 22 requisitions, $175,233.91, 6 contracts.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Wk2btL3DmVXUeNxgGiMYCy
</commit_message>
<xml_diff>
--- a/outputs/Exhibit_B_Verified_Conversions_JHK3.xlsx
+++ b/outputs/Exhibit_B_Verified_Conversions_JHK3.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="170">
   <si>
     <t xml:space="preserve">EXHIBIT B SPEND VERIFIED AS MOVED TO AN AWARDED CONTRACT</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">THE ANSWER</t>
   </si>
   <si>
-    <t xml:space="preserve">Yes - 8 Exhibit B items moved onto an awarded contract this year, covering 22 requisitions and $175,233.91 of maverick spend. 6 of the 8 went to a competitively bid contract - the correct outcome. The other 2 left Exhibit B through an emergency or sole-source award.</t>
+    <t xml:space="preserve">Yes - 8 Exhibit B items moved onto an awarded contract this year, covering 22 requisitions and $175,233.91 of maverick spend. All 8 are wins: the spend is now under a contract vehicle with negotiated terms and an audit trail, instead of being authorized purchase by purchase as a contract exception. 6 were competitively bid; the remainder were awarded by sole source or emergency, which are legitimate procurement methods with their own justification process - not maverick spend.</t>
   </si>
   <si>
     <t xml:space="preserve">THE NUMBERS</t>
@@ -60,7 +60,7 @@
     <t xml:space="preserve">Individual Exhibit B requisitions that rolled into those items</t>
   </si>
   <si>
-    <t xml:space="preserve">Maverick spend converted</t>
+    <t xml:space="preserve">Maverick spend eliminated</t>
   </si>
   <si>
     <t xml:space="preserve">Exhibit B dollars now covered by an awarded contract</t>
@@ -72,16 +72,16 @@
     <t xml:space="preserve">Fewer than the item count - separate Exhibit B items can converge on one contract</t>
   </si>
   <si>
-    <t xml:space="preserve">Went COMPETITIVE (Bid)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Competitively bid - the procurement-correct destination</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Went non-competitive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Emergency or sole source - off Exhibit B, but not competitively sourced</t>
+    <t xml:space="preserve">   awarded by competitive bid</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Competitively solicited</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   awarded by sole source or emergency</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Also a contract vehicle - justified, documented, auditable. Still a win</t>
   </si>
   <si>
     <t xml:space="preserve">Proven by requisition ID</t>
@@ -111,6 +111,12 @@
     <t xml:space="preserve">No matching requisition number, but the same vendor holds the new contract, the commodity descriptions overlap, and the award is dated after the Exhibit B request. Strong, but one step softer than an ID match - the similarity score is shown so it can be judged individually.</t>
   </si>
   <si>
+    <t xml:space="preserve">Award method is shown as information, not as a pass or fail</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every item listed is a win - the spend left Exhibit B and is now on a contract. The award method is reported because it tells you how the contract was procured, but a sole-source or emergency award is a legitimate, documented procurement vehicle. It is not maverick spend.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Timing test applied to every row</t>
   </si>
   <si>
@@ -126,7 +132,7 @@
     <t xml:space="preserve">VERIFIED CONVERSIONS - MAVERICK SPEND NOW UNDER CONTRACT</t>
   </si>
   <si>
-    <t xml:space="preserve">Each row is one Exhibit B item proven to have moved onto an awarded contract. The Proof column states the evidence.</t>
+    <t xml:space="preserve">Each row is one Exhibit B item proven to have moved onto an awarded contract - all are wins. The Proof column states the evidence.</t>
   </si>
   <si>
     <t xml:space="preserve">EXHIBIT B SIDE</t>
@@ -162,10 +168,7 @@
     <t xml:space="preserve">Award Date</t>
   </si>
   <si>
-    <t xml:space="preserve">Award Type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Competitive?</t>
+    <t xml:space="preserve">Award Method</t>
   </si>
   <si>
     <t xml:space="preserve">Proof</t>
@@ -186,9 +189,6 @@
     <t xml:space="preserve">EMERGENCY</t>
   </si>
   <si>
-    <t xml:space="preserve">NO</t>
-  </si>
-  <si>
     <t xml:space="preserve">DCASE submitted a new contract request for RENTAL AND MAINTENANCE OF PORTABLE CHEMICAL TOILETS,</t>
   </si>
   <si>
@@ -201,9 +201,6 @@
     <t xml:space="preserve">BID</t>
   </si>
   <si>
-    <t xml:space="preserve">YES</t>
-  </si>
-  <si>
     <t xml:space="preserve">Vendor + commodity match (0.64)</t>
   </si>
   <si>
@@ -471,7 +468,7 @@
     <t xml:space="preserve">Procurement Type</t>
   </si>
   <si>
-    <t xml:space="preserve">Competitive</t>
+    <t xml:space="preserve">Contract Type</t>
   </si>
   <si>
     <t xml:space="preserve">1232177</t>
@@ -483,6 +480,9 @@
     <t xml:space="preserve">85 - CHICAGO DEPARTMENT OF AVIATION</t>
   </si>
   <si>
+    <t xml:space="preserve">WORK SERV-AVIATION</t>
+  </si>
+  <si>
     <t xml:space="preserve">1321639</t>
   </si>
   <si>
@@ -492,6 +492,9 @@
     <t xml:space="preserve">41 - CHICAGO DEPARTMENT OF PUBLIC HEALTH</t>
   </si>
   <si>
+    <t xml:space="preserve">PRO SERV CONSULTING $250,000orABOVE</t>
+  </si>
+  <si>
     <t xml:space="preserve">1276708C</t>
   </si>
   <si>
@@ -501,6 +504,9 @@
     <t xml:space="preserve">35 - DEPARTMENT OF PROCUREMENT SERVICES</t>
   </si>
   <si>
+    <t xml:space="preserve">WORK SERVICES-SMALL ORDERS</t>
+  </si>
+  <si>
     <t xml:space="preserve">1334021</t>
   </si>
   <si>
@@ -508,6 +514,9 @@
   </si>
   <si>
     <t xml:space="preserve">38 - DEPARTMENT OF FLEET AND FACILITY MANAGEMENT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WORK SERVICES / FACILITIES MAINT.</t>
   </si>
   <si>
     <t xml:space="preserve">1303484</t>
@@ -535,7 +544,7 @@
     <numFmt numFmtId="166" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="167" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="17">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -628,14 +637,6 @@
     <font>
       <i val="true"/>
       <sz val="9"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <b val="true"/>
-      <sz val="9"/>
-      <color rgb="FFB26B00"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -769,7 +770,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -874,31 +875,23 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="14" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="16" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -932,7 +925,7 @@
       <rgbColor rgb="FF800000"/>
       <rgbColor rgb="FF1E7B34"/>
       <rgbColor rgb="FF000080"/>
-      <rgbColor rgb="FFB26B00"/>
+      <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FFBFBFBF"/>
@@ -1162,7 +1155,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1274,7 +1267,7 @@
         <v>16</v>
       </c>
       <c r="C14" s="8" t="n">
-        <f aca="false">COUNTIF('Verified Conversions'!$K$6:$K$13,"YES")</f>
+        <f aca="false">COUNTIF('Verified Conversions'!$J$6:$J$13,"BID")</f>
         <v>6</v>
       </c>
       <c r="D14" s="9" t="s">
@@ -1286,7 +1279,7 @@
         <v>18</v>
       </c>
       <c r="C15" s="8" t="n">
-        <f aca="false">COUNTIF('Verified Conversions'!$K$6:$K$13,"NO")</f>
+        <f aca="false">COUNTA('Verified Conversions'!$J$6:$J$13)-COUNTIF('Verified Conversions'!$J$6:$J$13,"BID")</f>
         <v>2</v>
       </c>
       <c r="D15" s="9" t="s">
@@ -1298,7 +1291,7 @@
         <v>20</v>
       </c>
       <c r="C16" s="8" t="n">
-        <f aca="false">COUNTIF('Verified Conversions'!$L$6:$L$13,"Requisition ID link")</f>
+        <f aca="false">COUNTIF('Verified Conversions'!$K$6:$K$13,"Requisition ID link")</f>
         <v>6</v>
       </c>
       <c r="D16" s="9" t="s">
@@ -1310,7 +1303,7 @@
         <v>22</v>
       </c>
       <c r="C17" s="8" t="n">
-        <f aca="false">COUNTA('Verified Conversions'!$L$6:$L$13)-COUNTIF('Verified Conversions'!$L$6:$L$13,"Requisition ID link")</f>
+        <f aca="false">COUNTA('Verified Conversions'!$K$6:$K$13)-COUNTIF('Verified Conversions'!$K$6:$K$13,"Requisition ID link")</f>
         <v>2</v>
       </c>
       <c r="D17" s="9" t="s">
@@ -1349,32 +1342,42 @@
       </c>
       <c r="D22" s="12"/>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="13" t="s">
+    <row r="23" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B23" s="11" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B25" s="14" t="s">
+      <c r="C23" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C25" s="14"/>
-      <c r="D25" s="14"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="14"/>
+      <c r="D23" s="12"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B25" s="13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B26" s="14" t="s">
+        <v>34</v>
+      </c>
       <c r="C26" s="14"/>
       <c r="D26" s="14"/>
     </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B27" s="14"/>
+      <c r="C27" s="14"/>
+      <c r="D27" s="14"/>
+    </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B5:D6"/>
     <mergeCell ref="C20:D20"/>
     <mergeCell ref="C21:D21"/>
     <mergeCell ref="C22:D22"/>
-    <mergeCell ref="B25:D26"/>
+    <mergeCell ref="C23:D23"/>
+    <mergeCell ref="B26:D27"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1391,7 +1394,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:L14"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1403,14 +1406,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="12" min="12" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="30"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1422,11 +1424,10 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1438,11 +1439,10 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B4" s="15"/>
       <c r="C4" s="15"/>
@@ -1450,50 +1450,46 @@
       <c r="E4" s="15"/>
       <c r="F4" s="15"/>
       <c r="G4" s="16" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="H4" s="16"/>
       <c r="I4" s="16"/>
       <c r="J4" s="16"/>
       <c r="K4" s="16"/>
-      <c r="L4" s="16"/>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I5" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K5" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="L5" s="6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1501,10 +1497,10 @@
         <v>1</v>
       </c>
       <c r="B6" s="18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D6" s="17" t="n">
         <v>6</v>
@@ -1516,21 +1512,18 @@
         <v>46045</v>
       </c>
       <c r="G6" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H6" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I6" s="20" t="n">
         <v>46203</v>
       </c>
-      <c r="J6" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="K6" s="21" t="s">
+      <c r="J6" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="L6" s="18" t="s">
+      <c r="K6" s="18" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1542,7 +1535,7 @@
         <v>55</v>
       </c>
       <c r="C7" s="22" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D7" s="22" t="n">
         <v>3</v>
@@ -1562,14 +1555,11 @@
       <c r="I7" s="25" t="n">
         <v>46203</v>
       </c>
-      <c r="J7" s="22" t="s">
+      <c r="J7" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="K7" s="26" t="s">
+      <c r="K7" s="23" t="s">
         <v>59</v>
-      </c>
-      <c r="L7" s="23" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1577,10 +1567,10 @@
         <v>3</v>
       </c>
       <c r="B8" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="17" t="s">
         <v>61</v>
-      </c>
-      <c r="C8" s="17" t="s">
-        <v>62</v>
       </c>
       <c r="D8" s="17" t="n">
         <v>1</v>
@@ -1592,21 +1582,18 @@
         <v>46216</v>
       </c>
       <c r="G8" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="H8" s="17" t="s">
         <v>63</v>
-      </c>
-      <c r="H8" s="17" t="s">
-        <v>64</v>
       </c>
       <c r="I8" s="20" t="n">
         <v>46229</v>
       </c>
-      <c r="J8" s="17" t="s">
+      <c r="J8" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="K8" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="L8" s="18" t="s">
+      <c r="K8" s="18" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1615,10 +1602,10 @@
         <v>4</v>
       </c>
       <c r="B9" s="23" t="s">
+        <v>64</v>
+      </c>
+      <c r="C9" s="22" t="s">
         <v>65</v>
-      </c>
-      <c r="C9" s="22" t="s">
-        <v>66</v>
       </c>
       <c r="D9" s="22" t="n">
         <v>3</v>
@@ -1630,21 +1617,18 @@
         <v>46119</v>
       </c>
       <c r="G9" s="22" t="s">
+        <v>66</v>
+      </c>
+      <c r="H9" s="22" t="s">
         <v>67</v>
-      </c>
-      <c r="H9" s="22" t="s">
-        <v>68</v>
       </c>
       <c r="I9" s="25" t="n">
         <v>46220</v>
       </c>
-      <c r="J9" s="22" t="s">
-        <v>69</v>
-      </c>
-      <c r="K9" s="28" t="s">
-        <v>54</v>
-      </c>
-      <c r="L9" s="23" t="s">
+      <c r="J9" s="26" t="s">
+        <v>68</v>
+      </c>
+      <c r="K9" s="23" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1653,10 +1637,10 @@
         <v>5</v>
       </c>
       <c r="B10" s="18" t="s">
+        <v>69</v>
+      </c>
+      <c r="C10" s="17" t="s">
         <v>70</v>
-      </c>
-      <c r="C10" s="17" t="s">
-        <v>71</v>
       </c>
       <c r="D10" s="17" t="n">
         <v>2</v>
@@ -1676,13 +1660,10 @@
       <c r="I10" s="20" t="n">
         <v>46203</v>
       </c>
-      <c r="J10" s="17" t="s">
+      <c r="J10" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="K10" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="L10" s="18" t="s">
+      <c r="K10" s="18" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1691,10 +1672,10 @@
         <v>6</v>
       </c>
       <c r="B11" s="23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C11" s="22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D11" s="22" t="n">
         <v>2</v>
@@ -1706,21 +1687,18 @@
         <v>46058</v>
       </c>
       <c r="G11" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="H11" s="22" t="s">
         <v>73</v>
-      </c>
-      <c r="H11" s="22" t="s">
-        <v>74</v>
       </c>
       <c r="I11" s="25" t="n">
         <v>46106</v>
       </c>
-      <c r="J11" s="22" t="s">
+      <c r="J11" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="K11" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="L11" s="23" t="s">
+      <c r="K11" s="23" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1729,10 +1707,10 @@
         <v>7</v>
       </c>
       <c r="B12" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="C12" s="17" t="s">
         <v>75</v>
-      </c>
-      <c r="C12" s="17" t="s">
-        <v>76</v>
       </c>
       <c r="D12" s="17" t="n">
         <v>4</v>
@@ -1752,14 +1730,11 @@
       <c r="I12" s="20" t="n">
         <v>46203</v>
       </c>
-      <c r="J12" s="17" t="s">
+      <c r="J12" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="K12" s="27" t="s">
-        <v>59</v>
-      </c>
-      <c r="L12" s="18" t="s">
-        <v>77</v>
+      <c r="K12" s="18" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1767,10 +1742,10 @@
         <v>8</v>
       </c>
       <c r="B13" s="23" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C13" s="22" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D13" s="22" t="n">
         <v>1</v>
@@ -1782,52 +1757,48 @@
         <v>46036</v>
       </c>
       <c r="G13" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="H13" s="22" t="s">
         <v>79</v>
-      </c>
-      <c r="H13" s="22" t="s">
-        <v>80</v>
       </c>
       <c r="I13" s="25" t="n">
         <v>46063</v>
       </c>
-      <c r="J13" s="22" t="s">
+      <c r="J13" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="K13" s="26" t="s">
-        <v>59</v>
-      </c>
-      <c r="L13" s="23" t="s">
+      <c r="K13" s="23" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="29"/>
-      <c r="B14" s="29" t="s">
-        <v>81</v>
-      </c>
-      <c r="C14" s="29"/>
-      <c r="D14" s="30" t="n">
+      <c r="A14" s="27"/>
+      <c r="B14" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="27"/>
+      <c r="D14" s="28" t="n">
         <f aca="false">SUM(D6:D13)</f>
         <v>22</v>
       </c>
-      <c r="E14" s="31" t="n">
+      <c r="E14" s="29" t="n">
         <f aca="false">SUM(E6:E13)</f>
         <v>175233.91</v>
       </c>
-      <c r="F14" s="29"/>
-      <c r="G14" s="29"/>
-      <c r="H14" s="29"/>
-      <c r="I14" s="29"/>
-      <c r="J14" s="29"/>
-      <c r="K14" s="29"/>
-      <c r="L14" s="29"/>
+      <c r="F14" s="27"/>
+      <c r="G14" s="27"/>
+      <c r="H14" s="27"/>
+      <c r="I14" s="27"/>
+      <c r="J14" s="27"/>
+      <c r="K14" s="27"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
     <mergeCell ref="A4:F4"/>
-    <mergeCell ref="G4:L4"/>
+    <mergeCell ref="G4:K4"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1862,7 +1833,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1877,7 +1848,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1891,48 +1862,48 @@
       <c r="K2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32" t="s">
-        <v>84</v>
+      <c r="A4" s="30" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
+        <v>84</v>
+      </c>
+      <c r="B5" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B5" s="6" t="s">
+      <c r="C5" s="6" t="s">
         <v>86</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="D5" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="E5" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="D5" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="E5" s="6" t="s">
+      <c r="F5" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="F5" s="6" t="s">
+      <c r="G5" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="H5" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="H5" s="6" t="s">
+      <c r="I5" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="I5" s="6" t="s">
+      <c r="J5" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="J5" s="6" t="s">
+      <c r="K5" s="6" t="s">
         <v>93</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B6" s="17" t="n">
         <v>707665</v>
@@ -1941,33 +1912,33 @@
         <v>46058</v>
       </c>
       <c r="D6" s="17" t="s">
+        <v>95</v>
+      </c>
+      <c r="E6" s="17" t="s">
         <v>96</v>
       </c>
-      <c r="E6" s="17" t="s">
+      <c r="F6" s="18" t="s">
         <v>97</v>
-      </c>
-      <c r="F6" s="18" t="s">
-        <v>98</v>
       </c>
       <c r="G6" s="19" t="n">
         <v>0</v>
       </c>
       <c r="H6" s="18" t="s">
+        <v>98</v>
+      </c>
+      <c r="I6" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="I6" s="17" t="s">
+      <c r="J6" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="K6" s="18" t="s">
         <v>100</v>
-      </c>
-      <c r="J6" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="K6" s="18" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="22" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B7" s="22" t="n">
         <v>716927</v>
@@ -1976,33 +1947,33 @@
         <v>46080</v>
       </c>
       <c r="D7" s="22" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E7" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="F7" s="23" t="s">
         <v>102</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>103</v>
       </c>
       <c r="G7" s="24" t="n">
         <v>2394.34</v>
       </c>
       <c r="H7" s="23" t="s">
+        <v>98</v>
+      </c>
+      <c r="I7" s="22" t="s">
         <v>99</v>
       </c>
-      <c r="I7" s="22" t="s">
+      <c r="J7" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="K7" s="23" t="s">
         <v>100</v>
-      </c>
-      <c r="J7" s="22" t="s">
-        <v>73</v>
-      </c>
-      <c r="K7" s="23" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>739971</v>
@@ -2011,33 +1982,33 @@
         <v>46216</v>
       </c>
       <c r="D8" s="17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E8" s="17" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8" s="18" t="s">
         <v>105</v>
-      </c>
-      <c r="F8" s="18" t="s">
-        <v>106</v>
       </c>
       <c r="G8" s="19" t="n">
         <v>9315</v>
       </c>
       <c r="H8" s="18" t="s">
+        <v>106</v>
+      </c>
+      <c r="I8" s="17" t="s">
         <v>107</v>
       </c>
-      <c r="I8" s="17" t="s">
-        <v>108</v>
-      </c>
       <c r="J8" s="17" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="K8" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="22" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B9" s="22" t="n">
         <v>711725</v>
@@ -2046,33 +2017,33 @@
         <v>46052</v>
       </c>
       <c r="D9" s="22" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E9" s="22" t="s">
         <v>57</v>
       </c>
       <c r="F9" s="23" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="G9" s="24" t="n">
         <v>1250</v>
       </c>
       <c r="H9" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I9" s="22" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J9" s="22" t="s">
         <v>56</v>
       </c>
       <c r="K9" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B10" s="17" t="n">
         <v>716858</v>
@@ -2081,33 +2052,33 @@
         <v>46080</v>
       </c>
       <c r="D10" s="17" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E10" s="17" t="s">
         <v>57</v>
       </c>
       <c r="F10" s="18" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G10" s="19" t="n">
         <v>5917</v>
       </c>
       <c r="H10" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I10" s="17" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J10" s="17" t="s">
         <v>56</v>
       </c>
       <c r="K10" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="22" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B11" s="22" t="n">
         <v>708543</v>
@@ -2116,33 +2087,33 @@
         <v>46036</v>
       </c>
       <c r="D11" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="E11" s="22" t="s">
         <v>115</v>
       </c>
-      <c r="E11" s="22" t="s">
+      <c r="F11" s="23" t="s">
         <v>116</v>
-      </c>
-      <c r="F11" s="23" t="s">
-        <v>117</v>
       </c>
       <c r="G11" s="24" t="n">
         <v>450</v>
       </c>
       <c r="H11" s="23" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="I11" s="22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="J11" s="22" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="K11" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B12" s="17" t="n">
         <v>722898</v>
@@ -2151,33 +2122,33 @@
         <v>46119</v>
       </c>
       <c r="D12" s="17" t="s">
+        <v>119</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="F12" s="18" t="s">
         <v>120</v>
-      </c>
-      <c r="E12" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="F12" s="18" t="s">
-        <v>121</v>
       </c>
       <c r="G12" s="19" t="n">
         <v>1890.66</v>
       </c>
       <c r="H12" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I12" s="17" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J12" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K12" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B13" s="22" t="n">
         <v>734145</v>
@@ -2186,33 +2157,33 @@
         <v>46177</v>
       </c>
       <c r="D13" s="22" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E13" s="22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F13" s="23" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="G13" s="24" t="n">
         <v>2499</v>
       </c>
       <c r="H13" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I13" s="22" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J13" s="22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K13" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B14" s="17" t="n">
         <v>738810</v>
@@ -2221,33 +2192,33 @@
         <v>46212</v>
       </c>
       <c r="D14" s="17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E14" s="17" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="G14" s="19" t="n">
         <v>3819.14</v>
       </c>
       <c r="H14" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I14" s="17" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J14" s="17" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="K14" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B15" s="22" t="n">
         <v>709848</v>
@@ -2256,33 +2227,33 @@
         <v>46045</v>
       </c>
       <c r="D15" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="E15" s="22" t="s">
+        <v>53</v>
+      </c>
+      <c r="F15" s="23" t="s">
         <v>125</v>
-      </c>
-      <c r="E15" s="22" t="s">
-        <v>52</v>
-      </c>
-      <c r="F15" s="23" t="s">
-        <v>126</v>
       </c>
       <c r="G15" s="24" t="n">
         <v>1297.26</v>
       </c>
       <c r="H15" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I15" s="22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J15" s="22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K15" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B16" s="17" t="n">
         <v>709600</v>
@@ -2291,33 +2262,33 @@
         <v>46048</v>
       </c>
       <c r="D16" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="E16" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="18" t="s">
         <v>125</v>
-      </c>
-      <c r="E16" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="F16" s="18" t="s">
-        <v>126</v>
       </c>
       <c r="G16" s="19" t="n">
         <v>840</v>
       </c>
       <c r="H16" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I16" s="17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J16" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K16" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B17" s="22" t="n">
         <v>710068</v>
@@ -2326,33 +2297,33 @@
         <v>46048</v>
       </c>
       <c r="D17" s="22" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E17" s="22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F17" s="23" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="G17" s="24" t="n">
         <v>18010.22</v>
       </c>
       <c r="H17" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I17" s="22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J17" s="22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K17" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B18" s="17" t="n">
         <v>718284</v>
@@ -2361,33 +2332,33 @@
         <v>46097</v>
       </c>
       <c r="D18" s="17" t="s">
+        <v>124</v>
+      </c>
+      <c r="E18" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="F18" s="18" t="s">
         <v>125</v>
-      </c>
-      <c r="E18" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="F18" s="18" t="s">
-        <v>126</v>
       </c>
       <c r="G18" s="19" t="n">
         <v>18935.29</v>
       </c>
       <c r="H18" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I18" s="17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J18" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K18" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="22" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B19" s="22" t="n">
         <v>728515</v>
@@ -2396,33 +2367,33 @@
         <v>46146</v>
       </c>
       <c r="D19" s="22" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E19" s="22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F19" s="23" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="G19" s="24" t="n">
         <v>89734.76</v>
       </c>
       <c r="H19" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I19" s="22" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J19" s="22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K19" s="23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B20" s="17" t="n">
         <v>730529</v>
@@ -2431,33 +2402,33 @@
         <v>46161</v>
       </c>
       <c r="D20" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E20" s="17" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="F20" s="18" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G20" s="19" t="n">
         <v>3458.74</v>
       </c>
       <c r="H20" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I20" s="17" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="J20" s="17" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="K20" s="18" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="22" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B21" s="22" t="n">
         <v>711517</v>
@@ -2466,33 +2437,33 @@
         <v>46052</v>
       </c>
       <c r="D21" s="22" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E21" s="22" t="s">
         <v>57</v>
       </c>
       <c r="F21" s="23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G21" s="24" t="n">
         <v>7750</v>
       </c>
       <c r="H21" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I21" s="22" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J21" s="22" t="s">
         <v>56</v>
       </c>
       <c r="K21" s="23" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B22" s="17" t="n">
         <v>711510</v>
@@ -2501,33 +2472,33 @@
         <v>46052</v>
       </c>
       <c r="D22" s="17" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E22" s="17" t="s">
         <v>57</v>
       </c>
       <c r="F22" s="18" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G22" s="19" t="n">
         <v>6700</v>
       </c>
       <c r="H22" s="18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I22" s="17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J22" s="17" t="s">
         <v>56</v>
       </c>
       <c r="K22" s="18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="22" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B23" s="22" t="n">
         <v>721747</v>
@@ -2536,33 +2507,33 @@
         <v>46107</v>
       </c>
       <c r="D23" s="22" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E23" s="22" t="s">
         <v>57</v>
       </c>
       <c r="F23" s="23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="G23" s="24" t="n">
         <v>247.5</v>
       </c>
       <c r="H23" s="23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="I23" s="22" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="J23" s="22" t="s">
         <v>56</v>
       </c>
       <c r="K23" s="23" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B24" s="17" t="n">
         <v>708558</v>
@@ -2571,33 +2542,33 @@
         <v>46038</v>
       </c>
       <c r="D24" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E24" s="17" t="s">
         <v>57</v>
       </c>
       <c r="F24" s="18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G24" s="19" t="n">
         <v>250</v>
       </c>
       <c r="H24" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="I24" s="17" t="s">
         <v>137</v>
-      </c>
-      <c r="I24" s="17" t="s">
-        <v>138</v>
       </c>
       <c r="J24" s="17" t="s">
         <v>56</v>
       </c>
       <c r="K24" s="18" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B25" s="22" t="n">
         <v>716043</v>
@@ -2606,33 +2577,33 @@
         <v>46078</v>
       </c>
       <c r="D25" s="22" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E25" s="22" t="s">
         <v>57</v>
       </c>
       <c r="F25" s="23" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G25" s="24" t="n">
         <v>225</v>
       </c>
       <c r="H25" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="I25" s="22" t="s">
         <v>137</v>
-      </c>
-      <c r="I25" s="22" t="s">
-        <v>138</v>
       </c>
       <c r="J25" s="22" t="s">
         <v>56</v>
       </c>
       <c r="K25" s="23" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="17" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B26" s="17" t="n">
         <v>716047</v>
@@ -2641,33 +2612,33 @@
         <v>46078</v>
       </c>
       <c r="D26" s="17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E26" s="17" t="s">
         <v>57</v>
       </c>
       <c r="F26" s="18" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G26" s="19" t="n">
         <v>250</v>
       </c>
       <c r="H26" s="18" t="s">
+        <v>136</v>
+      </c>
+      <c r="I26" s="17" t="s">
         <v>137</v>
-      </c>
-      <c r="I26" s="17" t="s">
-        <v>138</v>
       </c>
       <c r="J26" s="17" t="s">
         <v>56</v>
       </c>
       <c r="K26" s="18" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="22" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B27" s="22" t="n">
         <v>722165</v>
@@ -2676,91 +2647,91 @@
         <v>46118</v>
       </c>
       <c r="D27" s="22" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E27" s="22" t="s">
         <v>57</v>
       </c>
       <c r="F27" s="23" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G27" s="24" t="n">
         <v>0</v>
       </c>
       <c r="H27" s="23" t="s">
+        <v>136</v>
+      </c>
+      <c r="I27" s="22" t="s">
         <v>137</v>
-      </c>
-      <c r="I27" s="22" t="s">
-        <v>138</v>
       </c>
       <c r="J27" s="22" t="s">
         <v>56</v>
       </c>
       <c r="K27" s="23" t="s">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="31"/>
+      <c r="B28" s="31"/>
+      <c r="C28" s="31"/>
+      <c r="D28" s="31"/>
+      <c r="E28" s="31"/>
+      <c r="F28" s="31" t="s">
         <v>139</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="33"/>
-      <c r="B28" s="33"/>
-      <c r="C28" s="33"/>
-      <c r="D28" s="33"/>
-      <c r="E28" s="33"/>
-      <c r="F28" s="33" t="s">
-        <v>140</v>
-      </c>
-      <c r="G28" s="34" t="n">
+      <c r="G28" s="32" t="n">
         <f aca="false">SUM(G6:G27)</f>
         <v>175233.91</v>
       </c>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="33"/>
+      <c r="H28" s="31"/>
+      <c r="I28" s="31"/>
+      <c r="J28" s="31"/>
+      <c r="K28" s="31"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="32" t="s">
-        <v>141</v>
+      <c r="A30" s="30" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="B31" s="6" t="s">
+      <c r="C31" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="C31" s="6" t="s">
+      <c r="D31" s="6" t="s">
         <v>144</v>
       </c>
-      <c r="D31" s="6" t="s">
+      <c r="E31" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F31" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="E31" s="6" t="s">
-        <v>89</v>
-      </c>
-      <c r="F31" s="6" t="s">
+      <c r="G31" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>47</v>
+      </c>
+      <c r="I31" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="G31" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="H31" s="6" t="s">
-        <v>45</v>
-      </c>
-      <c r="I31" s="6" t="s">
+      <c r="J31" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="J31" s="6" t="s">
+      <c r="K31" s="6" t="s">
         <v>148</v>
-      </c>
-      <c r="K31" s="6" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B32" s="17" t="n">
         <v>329774</v>
@@ -2769,16 +2740,16 @@
         <v>530823</v>
       </c>
       <c r="D32" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="E32" s="18" t="s">
         <v>150</v>
       </c>
-      <c r="E32" s="18" t="s">
+      <c r="F32" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="G32" s="17" t="s">
         <v>151</v>
-      </c>
-      <c r="F32" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="G32" s="17" t="s">
-        <v>152</v>
       </c>
       <c r="H32" s="20" t="n">
         <v>46106</v>
@@ -2790,12 +2761,12 @@
         <v>58</v>
       </c>
       <c r="K32" s="17" t="s">
-        <v>59</v>
+        <v>152</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="22" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B33" s="22" t="n">
         <v>331452</v>
@@ -2810,7 +2781,7 @@
         <v>154</v>
       </c>
       <c r="F33" s="22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="G33" s="22" t="s">
         <v>155</v>
@@ -2822,15 +2793,15 @@
         <v>2100000</v>
       </c>
       <c r="J33" s="22" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="K33" s="22" t="s">
-        <v>54</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B34" s="17" t="n">
         <v>337037</v>
@@ -2839,16 +2810,16 @@
         <v>653063</v>
       </c>
       <c r="D34" s="17" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E34" s="18" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F34" s="17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="G34" s="17" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H34" s="20" t="n">
         <v>46063</v>
@@ -2860,12 +2831,12 @@
         <v>58</v>
       </c>
       <c r="K34" s="17" t="s">
-        <v>59</v>
+        <v>160</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="22" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B35" s="22" t="n">
         <v>342138</v>
@@ -2874,16 +2845,16 @@
         <v>690671</v>
       </c>
       <c r="D35" s="22" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="E35" s="23" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F35" s="22" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G35" s="22" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H35" s="25" t="n">
         <v>46203</v>
@@ -2892,10 +2863,10 @@
         <v>1000000</v>
       </c>
       <c r="J35" s="22" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="K35" s="22" t="s">
-        <v>54</v>
+        <v>164</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2909,16 +2880,16 @@
         <v>613315</v>
       </c>
       <c r="D36" s="17" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="E36" s="18" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F36" s="17" t="s">
         <v>57</v>
       </c>
       <c r="G36" s="17" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="H36" s="20" t="n">
         <v>46203</v>
@@ -2930,12 +2901,12 @@
         <v>58</v>
       </c>
       <c r="K36" s="17" t="s">
-        <v>59</v>
+        <v>164</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="22" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B37" s="22" t="n">
         <v>351919</v>
@@ -2944,16 +2915,16 @@
         <v>607558</v>
       </c>
       <c r="D37" s="22" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="E37" s="23" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F37" s="22" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="G37" s="22" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="H37" s="25" t="n">
         <v>46229</v>
@@ -2965,7 +2936,7 @@
         <v>58</v>
       </c>
       <c r="K37" s="22" t="s">
-        <v>59</v>
+        <v>152</v>
       </c>
     </row>
   </sheetData>

</xml_diff>